<commit_message>
data: publish 2026-09-08 daily operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-08-上海公交运营.xlsx
+++ b/data/export/2026-09-08-上海公交运营.xlsx
@@ -1502,11 +1502,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
+      <c r="Q13" t="n">
+        <v>1</v>
+      </c>
       <c r="R13" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S13" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1585,11 +1589,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
+      <c r="Q14" t="n">
+        <v>1</v>
+      </c>
       <c r="R14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S14" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1668,11 +1676,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
+      <c r="Q15" t="n">
+        <v>1</v>
+      </c>
       <c r="R15" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S15" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1751,11 +1763,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
+      <c r="Q16" t="n">
+        <v>1</v>
+      </c>
       <c r="R16" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S16" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1834,11 +1850,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
+      <c r="Q17" t="n">
+        <v>1</v>
+      </c>
       <c r="R17" t="n">
-        <v>0</v>
-      </c>
-      <c r="S17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S17" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1913,11 +1933,15 @@
         </is>
       </c>
       <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
+      <c r="Q18" t="n">
+        <v>1</v>
+      </c>
       <c r="R18" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S18" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1947,10 +1971,14 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>22:18</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -1963,17 +1991,17 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点近站ETA</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1983,12 +2011,20 @@
       </c>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>终点近站ETA推算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
+        <v>1</v>
+      </c>
       <c r="R19" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S19" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3131,7 +3167,7 @@
         </is>
       </c>
       <c r="Q33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R33" t="n">
         <v>1</v>
@@ -3218,7 +3254,7 @@
         </is>
       </c>
       <c r="Q34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R34" t="n">
         <v>1</v>
@@ -3305,7 +3341,7 @@
         </is>
       </c>
       <c r="Q35" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R35" t="n">
         <v>1</v>
@@ -3392,7 +3428,7 @@
         </is>
       </c>
       <c r="Q36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R36" t="n">
         <v>1</v>
@@ -3479,7 +3515,7 @@
         </is>
       </c>
       <c r="Q37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R37" t="n">
         <v>1</v>
@@ -3562,7 +3598,7 @@
         </is>
       </c>
       <c r="Q38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R38" t="n">
         <v>1</v>
@@ -3637,7 +3673,7 @@
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R39" t="n">
         <v>1</v>
@@ -3724,7 +3760,7 @@
         </is>
       </c>
       <c r="Q40" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R40" t="n">
         <v>1</v>
@@ -3811,7 +3847,7 @@
         </is>
       </c>
       <c r="Q41" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R41" t="n">
         <v>1</v>
@@ -3898,7 +3934,7 @@
         </is>
       </c>
       <c r="Q42" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R42" t="n">
         <v>1</v>
@@ -3985,7 +4021,7 @@
         </is>
       </c>
       <c r="Q43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R43" t="n">
         <v>1</v>
@@ -4072,7 +4108,7 @@
         </is>
       </c>
       <c r="Q44" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R44" t="n">
         <v>1</v>
@@ -4155,7 +4191,7 @@
         </is>
       </c>
       <c r="Q45" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R45" t="n">
         <v>1</v>
@@ -4230,7 +4266,7 @@
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R46" t="n">
         <v>1</v>
@@ -4554,7 +4590,7 @@
         </is>
       </c>
       <c r="Q50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R50" t="n">
         <v>1</v>
@@ -4641,7 +4677,7 @@
         </is>
       </c>
       <c r="Q51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R51" t="n">
         <v>1</v>
@@ -4724,7 +4760,7 @@
         </is>
       </c>
       <c r="Q52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R52" t="n">
         <v>1</v>
@@ -4811,7 +4847,7 @@
         </is>
       </c>
       <c r="Q53" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R53" t="n">
         <v>1</v>
@@ -4898,7 +4934,7 @@
         </is>
       </c>
       <c r="Q54" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R54" t="n">
         <v>1</v>
@@ -4985,7 +5021,7 @@
         </is>
       </c>
       <c r="Q55" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R55" t="n">
         <v>1</v>
@@ -5068,7 +5104,7 @@
         </is>
       </c>
       <c r="Q56" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R56" t="n">
         <v>1</v>
@@ -5155,7 +5191,7 @@
         </is>
       </c>
       <c r="Q57" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R57" t="n">
         <v>1</v>
@@ -5242,7 +5278,7 @@
         </is>
       </c>
       <c r="Q58" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R58" t="n">
         <v>1</v>
@@ -5329,7 +5365,7 @@
         </is>
       </c>
       <c r="Q59" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R59" t="n">
         <v>1</v>
@@ -5416,7 +5452,7 @@
         </is>
       </c>
       <c r="Q60" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R60" t="n">
         <v>1</v>
@@ -5503,7 +5539,7 @@
         </is>
       </c>
       <c r="Q61" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R61" t="n">
         <v>1</v>
@@ -5586,7 +5622,7 @@
         </is>
       </c>
       <c r="Q62" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R62" t="n">
         <v>1</v>
@@ -5661,7 +5697,7 @@
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr"/>
       <c r="Q63" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R63" t="n">
         <v>1</v>
@@ -5748,7 +5784,7 @@
         </is>
       </c>
       <c r="Q64" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R64" t="n">
         <v>1</v>
@@ -5835,7 +5871,7 @@
         </is>
       </c>
       <c r="Q65" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R65" t="n">
         <v>1</v>
@@ -5922,7 +5958,7 @@
         </is>
       </c>
       <c r="Q66" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R66" t="n">
         <v>1</v>
@@ -6009,7 +6045,7 @@
         </is>
       </c>
       <c r="Q67" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R67" t="n">
         <v>1</v>
@@ -6096,7 +6132,7 @@
         </is>
       </c>
       <c r="Q68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R68" t="n">
         <v>1</v>
@@ -6179,7 +6215,7 @@
         </is>
       </c>
       <c r="Q69" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R69" t="n">
         <v>1</v>
@@ -6254,7 +6290,7 @@
       <c r="O70" t="inlineStr"/>
       <c r="P70" t="inlineStr"/>
       <c r="Q70" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R70" t="n">
         <v>1</v>
@@ -6835,7 +6871,7 @@
         </is>
       </c>
       <c r="Q77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R77" t="n">
         <v>1</v>
@@ -6922,7 +6958,7 @@
         </is>
       </c>
       <c r="Q78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R78" t="n">
         <v>1</v>
@@ -7009,7 +7045,7 @@
         </is>
       </c>
       <c r="Q79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R79" t="n">
         <v>1</v>
@@ -7096,7 +7132,7 @@
         </is>
       </c>
       <c r="Q80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R80" t="n">
         <v>1</v>
@@ -7183,7 +7219,7 @@
         </is>
       </c>
       <c r="Q81" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R81" t="n">
         <v>1</v>
@@ -7266,7 +7302,7 @@
       </c>
       <c r="P82" t="inlineStr"/>
       <c r="Q82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R82" t="n">
         <v>1</v>
@@ -7349,7 +7385,7 @@
         </is>
       </c>
       <c r="Q83" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R83" t="n">
         <v>1</v>
@@ -7424,7 +7460,7 @@
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr"/>
       <c r="Q84" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R84" t="n">
         <v>1</v>
@@ -8842,7 +8878,7 @@
       </c>
       <c r="P102" t="inlineStr"/>
       <c r="Q102" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R102" t="n">
         <v>1</v>
@@ -8925,7 +8961,7 @@
         </is>
       </c>
       <c r="Q103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R103" t="n">
         <v>1</v>
@@ -9012,7 +9048,7 @@
         </is>
       </c>
       <c r="Q104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R104" t="n">
         <v>1</v>
@@ -9095,7 +9131,7 @@
       </c>
       <c r="P105" t="inlineStr"/>
       <c r="Q105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R105" t="n">
         <v>1</v>
@@ -10347,7 +10383,7 @@
         </is>
       </c>
       <c r="Q121" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R121" t="n">
         <v>2</v>
@@ -10430,7 +10466,7 @@
         </is>
       </c>
       <c r="Q122" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R122" t="n">
         <v>2</v>
@@ -10513,7 +10549,7 @@
         </is>
       </c>
       <c r="Q123" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R123" t="n">
         <v>2</v>
@@ -10600,7 +10636,7 @@
         </is>
       </c>
       <c r="Q124" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R124" t="n">
         <v>2</v>
@@ -10687,7 +10723,7 @@
         </is>
       </c>
       <c r="Q125" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R125" t="n">
         <v>2</v>
@@ -10762,7 +10798,7 @@
       <c r="O126" t="inlineStr"/>
       <c r="P126" t="inlineStr"/>
       <c r="Q126" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R126" t="n">
         <v>2</v>
@@ -10849,7 +10885,7 @@
         </is>
       </c>
       <c r="Q127" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R127" t="n">
         <v>2</v>
@@ -10932,7 +10968,7 @@
         </is>
       </c>
       <c r="Q128" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R128" t="n">
         <v>2</v>
@@ -11019,7 +11055,7 @@
         </is>
       </c>
       <c r="Q129" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R129" t="n">
         <v>2</v>
@@ -11106,7 +11142,7 @@
         </is>
       </c>
       <c r="Q130" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R130" t="n">
         <v>2</v>
@@ -11189,7 +11225,7 @@
         </is>
       </c>
       <c r="Q131" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R131" t="n">
         <v>2</v>
@@ -11276,7 +11312,7 @@
         </is>
       </c>
       <c r="Q132" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R132" t="n">
         <v>1</v>
@@ -11359,7 +11395,7 @@
       </c>
       <c r="P133" t="inlineStr"/>
       <c r="Q133" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R133" t="n">
         <v>1</v>
@@ -11446,7 +11482,7 @@
         </is>
       </c>
       <c r="Q134" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R134" t="n">
         <v>1</v>
@@ -11529,7 +11565,7 @@
         </is>
       </c>
       <c r="Q135" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R135" t="n">
         <v>1</v>
@@ -11612,7 +11648,7 @@
         </is>
       </c>
       <c r="Q136" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R136" t="n">
         <v>3</v>
@@ -11699,7 +11735,7 @@
         </is>
       </c>
       <c r="Q137" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R137" t="n">
         <v>3</v>
@@ -11782,7 +11818,7 @@
         </is>
       </c>
       <c r="Q138" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R138" t="n">
         <v>3</v>
@@ -11869,7 +11905,7 @@
         </is>
       </c>
       <c r="Q139" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R139" t="n">
         <v>3</v>
@@ -11956,7 +11992,7 @@
         </is>
       </c>
       <c r="Q140" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R140" t="n">
         <v>3</v>
@@ -12039,7 +12075,7 @@
         </is>
       </c>
       <c r="Q141" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R141" t="n">
         <v>3</v>
@@ -12122,7 +12158,7 @@
       </c>
       <c r="P142" t="inlineStr"/>
       <c r="Q142" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R142" t="n">
         <v>1</v>
@@ -12209,7 +12245,7 @@
         </is>
       </c>
       <c r="Q143" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R143" t="n">
         <v>1</v>
@@ -12296,7 +12332,7 @@
         </is>
       </c>
       <c r="Q144" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R144" t="n">
         <v>1</v>
@@ -12379,7 +12415,7 @@
         </is>
       </c>
       <c r="Q145" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R145" t="n">
         <v>1</v>
@@ -12466,7 +12502,7 @@
         </is>
       </c>
       <c r="Q146" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R146" t="n">
         <v>1</v>
@@ -12553,7 +12589,7 @@
         </is>
       </c>
       <c r="Q147" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R147" t="n">
         <v>1</v>
@@ -12640,7 +12676,7 @@
         </is>
       </c>
       <c r="Q148" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R148" t="n">
         <v>1</v>
@@ -12723,7 +12759,7 @@
         </is>
       </c>
       <c r="Q149" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R149" t="n">
         <v>1</v>
@@ -13370,11 +13406,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q157" t="inlineStr"/>
+      <c r="Q157" t="n">
+        <v>5</v>
+      </c>
       <c r="R157" t="n">
-        <v>0</v>
-      </c>
-      <c r="S157" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S157" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -13453,11 +13493,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q158" t="inlineStr"/>
+      <c r="Q158" t="n">
+        <v>5</v>
+      </c>
       <c r="R158" t="n">
-        <v>0</v>
-      </c>
-      <c r="S158" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S158" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -13493,12 +13537,12 @@
       <c r="G159" t="inlineStr"/>
       <c r="H159" t="inlineStr">
         <is>
-          <t>全程车</t>
+          <t>运行异常待查</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>未发现可靠中途折返证据</t>
+          <t>存在方向切换，但未达到提前反向80%判据</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
@@ -13521,14 +13565,26 @@
           <t>07:10</t>
         </is>
       </c>
-      <c r="N159" t="inlineStr"/>
-      <c r="O159" t="inlineStr"/>
+      <c r="N159" s="1" t="inlineStr">
+        <is>
+          <t>长岛路张杨北路</t>
+        </is>
+      </c>
+      <c r="O159" s="1" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
       <c r="P159" t="inlineStr"/>
-      <c r="Q159" t="inlineStr"/>
+      <c r="Q159" t="n">
+        <v>5</v>
+      </c>
       <c r="R159" t="n">
-        <v>0</v>
-      </c>
-      <c r="S159" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S159" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -13558,10 +13614,14 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G160" t="inlineStr"/>
+          <t>22:38</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
       <c r="H160" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -13574,17 +13634,17 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>多次终点ETA一致</t>
         </is>
       </c>
       <c r="L160" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M160" t="inlineStr">
@@ -13594,12 +13654,20 @@
       </c>
       <c r="N160" t="inlineStr"/>
       <c r="O160" t="inlineStr"/>
-      <c r="P160" t="inlineStr"/>
-      <c r="Q160" t="inlineStr"/>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>多次终点ETA一致推算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="Q160" t="n">
+        <v>5</v>
+      </c>
       <c r="R160" t="n">
-        <v>0</v>
-      </c>
-      <c r="S160" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S160" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -13675,7 +13743,7 @@
       </c>
       <c r="P161" t="inlineStr"/>
       <c r="Q161" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R161" t="n">
         <v>1</v>
@@ -13762,7 +13830,7 @@
         </is>
       </c>
       <c r="Q162" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R162" t="n">
         <v>1</v>
@@ -13845,7 +13913,7 @@
         </is>
       </c>
       <c r="Q163" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R163" t="n">
         <v>1</v>
@@ -13920,7 +13988,7 @@
       <c r="O164" t="inlineStr"/>
       <c r="P164" t="inlineStr"/>
       <c r="Q164" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R164" t="n">
         <v>1</v>
@@ -14007,13 +14075,13 @@
         </is>
       </c>
       <c r="Q165" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R165" t="n">
         <v>1</v>
       </c>
       <c r="S165" t="n">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="166">
@@ -14094,13 +14162,13 @@
         </is>
       </c>
       <c r="Q166" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R166" t="n">
         <v>1</v>
       </c>
       <c r="S166" t="n">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="167">
@@ -14131,37 +14199,33 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>20:31</t>
-        </is>
-      </c>
-      <c r="G167" t="inlineStr">
-        <is>
-          <t>131</t>
-        </is>
-      </c>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr"/>
       <c r="H167" t="inlineStr">
         <is>
-          <t>全程车</t>
+          <t>运行异常待查</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>未发现可靠中途折返证据</t>
+          <t>末次同向观测已进入线路末段，存在终点漏采可能</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>末次终点ETA</t>
+          <t>证据不足</t>
         </is>
       </c>
       <c r="L167" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="M167" t="inlineStr">
@@ -14169,21 +14233,29 @@
           <t>07:24</t>
         </is>
       </c>
-      <c r="N167" t="inlineStr"/>
-      <c r="O167" t="inlineStr"/>
+      <c r="N167" s="1" t="inlineStr">
+        <is>
+          <t>康弘路康佳路（康桥卫生中心）</t>
+        </is>
+      </c>
+      <c r="O167" s="1" t="inlineStr">
+        <is>
+          <t>20:24</t>
+        </is>
+      </c>
       <c r="P167" t="inlineStr">
         <is>
-          <t>末次终点ETA推算，约±10分钟</t>
+          <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
       <c r="Q167" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R167" t="n">
         <v>1</v>
       </c>
       <c r="S167" t="n">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="168">
@@ -14214,10 +14286,14 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G168" t="inlineStr"/>
+          <t>22:58</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
       <c r="H168" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -14230,17 +14306,17 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>末次终点ETA</t>
         </is>
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M168" t="inlineStr">
@@ -14250,15 +14326,19 @@
       </c>
       <c r="N168" t="inlineStr"/>
       <c r="O168" t="inlineStr"/>
-      <c r="P168" t="inlineStr"/>
+      <c r="P168" t="inlineStr">
+        <is>
+          <t>末次终点ETA推算，约±15分钟</t>
+        </is>
+      </c>
       <c r="Q168" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R168" t="n">
         <v>1</v>
       </c>
       <c r="S168" t="n">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="169">
@@ -14825,7 +14905,7 @@
         </is>
       </c>
       <c r="Q175" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R175" t="n">
         <v>1</v>
@@ -14912,7 +14992,7 @@
         </is>
       </c>
       <c r="Q176" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R176" t="n">
         <v>1</v>
@@ -14995,7 +15075,7 @@
       </c>
       <c r="P177" t="inlineStr"/>
       <c r="Q177" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R177" t="n">
         <v>1</v>
@@ -15078,7 +15158,7 @@
         </is>
       </c>
       <c r="Q178" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R178" t="n">
         <v>1</v>
@@ -15165,7 +15245,7 @@
         </is>
       </c>
       <c r="Q179" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R179" t="n">
         <v>1</v>
@@ -15248,7 +15328,7 @@
         </is>
       </c>
       <c r="Q180" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R180" t="n">
         <v>1</v>
@@ -15335,7 +15415,7 @@
         </is>
       </c>
       <c r="Q181" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R181" t="n">
         <v>1</v>
@@ -15422,7 +15502,7 @@
         </is>
       </c>
       <c r="Q182" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R182" t="n">
         <v>1</v>
@@ -15497,7 +15577,7 @@
       <c r="O183" t="inlineStr"/>
       <c r="P183" t="inlineStr"/>
       <c r="Q183" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R183" t="n">
         <v>1</v>
@@ -15900,7 +15980,7 @@
         </is>
       </c>
       <c r="Q188" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R188" t="n">
         <v>1</v>
@@ -15983,7 +16063,7 @@
         </is>
       </c>
       <c r="Q189" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R189" t="n">
         <v>1</v>
@@ -16070,7 +16150,7 @@
         </is>
       </c>
       <c r="Q190" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R190" t="n">
         <v>1</v>
@@ -16157,7 +16237,7 @@
         </is>
       </c>
       <c r="Q191" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R191" t="n">
         <v>1</v>
@@ -16244,7 +16324,7 @@
         </is>
       </c>
       <c r="Q192" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R192" t="n">
         <v>1</v>
@@ -16327,7 +16407,7 @@
         </is>
       </c>
       <c r="Q193" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R193" t="n">
         <v>1</v>
@@ -16414,7 +16494,7 @@
         </is>
       </c>
       <c r="Q194" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R194" t="n">
         <v>1</v>
@@ -16497,7 +16577,7 @@
       </c>
       <c r="P195" t="inlineStr"/>
       <c r="Q195" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R195" t="n">
         <v>1</v>
@@ -17619,7 +17699,7 @@
         </is>
       </c>
       <c r="Q209" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R209" t="n">
         <v>2</v>
@@ -17706,7 +17786,7 @@
         </is>
       </c>
       <c r="Q210" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R210" t="n">
         <v>2</v>
@@ -17789,7 +17869,7 @@
         </is>
       </c>
       <c r="Q211" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R211" t="n">
         <v>2</v>
@@ -17876,7 +17956,7 @@
         </is>
       </c>
       <c r="Q212" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R212" t="n">
         <v>2</v>
@@ -17963,7 +18043,7 @@
         </is>
       </c>
       <c r="Q213" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R213" t="n">
         <v>2</v>
@@ -18050,7 +18130,7 @@
         </is>
       </c>
       <c r="Q214" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R214" t="n">
         <v>2</v>
@@ -18133,7 +18213,7 @@
         </is>
       </c>
       <c r="Q215" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R215" t="n">
         <v>2</v>
@@ -18208,7 +18288,7 @@
       <c r="O216" t="inlineStr"/>
       <c r="P216" t="inlineStr"/>
       <c r="Q216" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R216" t="n">
         <v>2</v>
@@ -18856,7 +18936,7 @@
         </is>
       </c>
       <c r="Q224" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R224" t="n">
         <v>1</v>
@@ -18943,7 +19023,7 @@
         </is>
       </c>
       <c r="Q225" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R225" t="n">
         <v>1</v>
@@ -19026,7 +19106,7 @@
       </c>
       <c r="P226" t="inlineStr"/>
       <c r="Q226" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R226" t="n">
         <v>1</v>
@@ -19109,7 +19189,7 @@
         </is>
       </c>
       <c r="Q227" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R227" t="n">
         <v>1</v>
@@ -19184,7 +19264,7 @@
       <c r="O228" t="inlineStr"/>
       <c r="P228" t="inlineStr"/>
       <c r="Q228" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R228" t="n">
         <v>1</v>
@@ -19267,7 +19347,7 @@
         </is>
       </c>
       <c r="Q229" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="R229" t="n">
         <v>1</v>
@@ -19354,7 +19434,7 @@
         </is>
       </c>
       <c r="Q230" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R230" t="n">
         <v>1</v>
@@ -19441,7 +19521,7 @@
         </is>
       </c>
       <c r="Q231" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R231" t="n">
         <v>1</v>
@@ -19528,7 +19608,7 @@
         </is>
       </c>
       <c r="Q232" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R232" t="n">
         <v>1</v>
@@ -19615,7 +19695,7 @@
         </is>
       </c>
       <c r="Q233" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R233" t="n">
         <v>1</v>
@@ -19702,7 +19782,7 @@
         </is>
       </c>
       <c r="Q234" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R234" t="n">
         <v>1</v>
@@ -19785,7 +19865,7 @@
         </is>
       </c>
       <c r="Q235" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R235" t="n">
         <v>1</v>
@@ -19860,7 +19940,7 @@
       <c r="O236" t="inlineStr"/>
       <c r="P236" t="inlineStr"/>
       <c r="Q236" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R236" t="n">
         <v>1</v>
@@ -20425,7 +20505,7 @@
       </c>
       <c r="P243" t="inlineStr"/>
       <c r="Q243" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R243" t="n">
         <v>1</v>
@@ -20508,7 +20588,7 @@
         </is>
       </c>
       <c r="Q244" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R244" t="n">
         <v>1</v>
@@ -20595,7 +20675,7 @@
         </is>
       </c>
       <c r="Q245" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R245" t="n">
         <v>1</v>
@@ -20670,7 +20750,7 @@
       <c r="O246" t="inlineStr"/>
       <c r="P246" t="inlineStr"/>
       <c r="Q246" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R246" t="n">
         <v>1</v>
@@ -20757,7 +20837,7 @@
         </is>
       </c>
       <c r="Q247" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R247" t="n">
         <v>1</v>
@@ -20840,7 +20920,7 @@
         </is>
       </c>
       <c r="Q248" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R248" t="n">
         <v>1</v>
@@ -20927,7 +21007,7 @@
         </is>
       </c>
       <c r="Q249" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R249" t="n">
         <v>1</v>
@@ -21014,7 +21094,7 @@
         </is>
       </c>
       <c r="Q250" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R250" t="n">
         <v>1</v>
@@ -21101,7 +21181,7 @@
         </is>
       </c>
       <c r="Q251" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R251" t="n">
         <v>1</v>
@@ -21188,7 +21268,7 @@
         </is>
       </c>
       <c r="Q252" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R252" t="n">
         <v>1</v>
@@ -21271,7 +21351,7 @@
       </c>
       <c r="P253" t="inlineStr"/>
       <c r="Q253" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R253" t="n">
         <v>1</v>
@@ -21346,7 +21426,7 @@
       <c r="O254" t="inlineStr"/>
       <c r="P254" t="inlineStr"/>
       <c r="Q254" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R254" t="n">
         <v>1</v>
@@ -21433,7 +21513,7 @@
         </is>
       </c>
       <c r="Q255" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R255" t="n">
         <v>1</v>
@@ -21520,7 +21600,7 @@
         </is>
       </c>
       <c r="Q256" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R256" t="n">
         <v>1</v>
@@ -21607,7 +21687,7 @@
         </is>
       </c>
       <c r="Q257" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R257" t="n">
         <v>1</v>
@@ -21694,7 +21774,7 @@
         </is>
       </c>
       <c r="Q258" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R258" t="n">
         <v>1</v>
@@ -21781,7 +21861,7 @@
         </is>
       </c>
       <c r="Q259" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R259" t="n">
         <v>1</v>
@@ -21864,7 +21944,7 @@
         </is>
       </c>
       <c r="Q260" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R260" t="n">
         <v>1</v>
@@ -21939,7 +22019,7 @@
       <c r="O261" t="inlineStr"/>
       <c r="P261" t="inlineStr"/>
       <c r="Q261" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R261" t="n">
         <v>1</v>
@@ -22021,11 +22101,15 @@
         </is>
       </c>
       <c r="P262" t="inlineStr"/>
-      <c r="Q262" t="inlineStr"/>
+      <c r="Q262" t="n">
+        <v>1</v>
+      </c>
       <c r="R262" t="n">
-        <v>0</v>
-      </c>
-      <c r="S262" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S262" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -22104,11 +22188,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q263" t="inlineStr"/>
+      <c r="Q263" t="n">
+        <v>1</v>
+      </c>
       <c r="R263" t="n">
-        <v>0</v>
-      </c>
-      <c r="S263" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S263" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -22187,11 +22275,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q264" t="inlineStr"/>
+      <c r="Q264" t="n">
+        <v>1</v>
+      </c>
       <c r="R264" t="n">
-        <v>0</v>
-      </c>
-      <c r="S264" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S264" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -22266,11 +22358,15 @@
         </is>
       </c>
       <c r="P265" t="inlineStr"/>
-      <c r="Q265" t="inlineStr"/>
+      <c r="Q265" t="n">
+        <v>1</v>
+      </c>
       <c r="R265" t="n">
-        <v>0</v>
-      </c>
-      <c r="S265" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S265" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -22300,10 +22396,14 @@
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G266" t="inlineStr"/>
+          <t>22:27</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
       <c r="H266" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -22316,17 +22416,17 @@
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>多次终点ETA一致</t>
         </is>
       </c>
       <c r="L266" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M266" t="inlineStr">
@@ -22336,12 +22436,20 @@
       </c>
       <c r="N266" t="inlineStr"/>
       <c r="O266" t="inlineStr"/>
-      <c r="P266" t="inlineStr"/>
-      <c r="Q266" t="inlineStr"/>
+      <c r="P266" t="inlineStr">
+        <is>
+          <t>多次终点ETA一致推算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="Q266" t="n">
+        <v>1</v>
+      </c>
       <c r="R266" t="n">
-        <v>0</v>
-      </c>
-      <c r="S266" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S266" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -22416,11 +22524,15 @@
         </is>
       </c>
       <c r="P267" t="inlineStr"/>
-      <c r="Q267" t="inlineStr"/>
+      <c r="Q267" t="n">
+        <v>3</v>
+      </c>
       <c r="R267" t="n">
-        <v>0</v>
-      </c>
-      <c r="S267" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S267" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -22499,11 +22611,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q268" t="inlineStr"/>
+      <c r="Q268" t="n">
+        <v>3</v>
+      </c>
       <c r="R268" t="n">
-        <v>0</v>
-      </c>
-      <c r="S268" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S268" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -22578,11 +22694,15 @@
         </is>
       </c>
       <c r="P269" t="inlineStr"/>
-      <c r="Q269" t="inlineStr"/>
+      <c r="Q269" t="n">
+        <v>3</v>
+      </c>
       <c r="R269" t="n">
-        <v>0</v>
-      </c>
-      <c r="S269" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S269" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -22657,11 +22777,15 @@
         </is>
       </c>
       <c r="P270" t="inlineStr"/>
-      <c r="Q270" t="inlineStr"/>
+      <c r="Q270" t="n">
+        <v>3</v>
+      </c>
       <c r="R270" t="n">
-        <v>0</v>
-      </c>
-      <c r="S270" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S270" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -22691,10 +22815,14 @@
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G271" t="inlineStr"/>
+          <t>23:03</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
       <c r="H271" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -22707,17 +22835,17 @@
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>多次终点ETA一致</t>
         </is>
       </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M271" t="inlineStr">
@@ -22727,12 +22855,20 @@
       </c>
       <c r="N271" t="inlineStr"/>
       <c r="O271" t="inlineStr"/>
-      <c r="P271" t="inlineStr"/>
-      <c r="Q271" t="inlineStr"/>
+      <c r="P271" t="inlineStr">
+        <is>
+          <t>多次终点ETA一致推算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="Q271" t="n">
+        <v>3</v>
+      </c>
       <c r="R271" t="n">
-        <v>0</v>
-      </c>
-      <c r="S271" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S271" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -22808,7 +22944,7 @@
       </c>
       <c r="P272" t="inlineStr"/>
       <c r="Q272" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R272" t="n">
         <v>1</v>
@@ -22891,7 +23027,7 @@
       </c>
       <c r="P273" t="inlineStr"/>
       <c r="Q273" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R273" t="n">
         <v>1</v>
@@ -22978,7 +23114,7 @@
         </is>
       </c>
       <c r="Q274" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R274" t="n">
         <v>1</v>
@@ -23065,7 +23201,7 @@
         </is>
       </c>
       <c r="Q275" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R275" t="n">
         <v>1</v>
@@ -23152,7 +23288,7 @@
         </is>
       </c>
       <c r="Q276" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R276" t="n">
         <v>1</v>
@@ -23235,7 +23371,7 @@
         </is>
       </c>
       <c r="Q277" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R277" t="n">
         <v>1</v>
@@ -23318,7 +23454,7 @@
       </c>
       <c r="P278" t="inlineStr"/>
       <c r="Q278" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="R278" t="n">
         <v>1</v>
@@ -23405,7 +23541,7 @@
         </is>
       </c>
       <c r="Q279" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="R279" t="n">
         <v>1</v>
@@ -23488,7 +23624,7 @@
         </is>
       </c>
       <c r="Q280" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="R280" t="n">
         <v>1</v>
@@ -23563,7 +23699,7 @@
       <c r="O281" t="inlineStr"/>
       <c r="P281" t="inlineStr"/>
       <c r="Q281" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="R281" t="n">
         <v>1</v>
@@ -23650,7 +23786,7 @@
         </is>
       </c>
       <c r="Q282" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R282" t="n">
         <v>1</v>
@@ -23737,7 +23873,7 @@
         </is>
       </c>
       <c r="Q283" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R283" t="n">
         <v>1</v>
@@ -23824,7 +23960,7 @@
         </is>
       </c>
       <c r="Q284" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R284" t="n">
         <v>1</v>
@@ -23907,7 +24043,7 @@
         </is>
       </c>
       <c r="Q285" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R285" t="n">
         <v>1</v>
@@ -23982,7 +24118,7 @@
       <c r="O286" t="inlineStr"/>
       <c r="P286" t="inlineStr"/>
       <c r="Q286" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R286" t="n">
         <v>1</v>
@@ -26031,7 +26167,7 @@
         </is>
       </c>
       <c r="Q12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R12" t="n">
         <v>2</v>
@@ -26118,7 +26254,7 @@
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R13" t="n">
         <v>2</v>
@@ -26201,7 +26337,7 @@
         </is>
       </c>
       <c r="Q14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R14" t="n">
         <v>2</v>
@@ -26288,7 +26424,7 @@
         </is>
       </c>
       <c r="Q15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R15" t="n">
         <v>2</v>
@@ -26375,7 +26511,7 @@
         </is>
       </c>
       <c r="Q16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R16" t="n">
         <v>2</v>
@@ -26462,7 +26598,7 @@
         </is>
       </c>
       <c r="Q17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R17" t="n">
         <v>2</v>
@@ -26545,7 +26681,7 @@
         </is>
       </c>
       <c r="Q18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R18" t="n">
         <v>2</v>
@@ -26620,7 +26756,7 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R19" t="n">
         <v>2</v>
@@ -27268,7 +27404,7 @@
         </is>
       </c>
       <c r="Q27" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R27" t="n">
         <v>1</v>
@@ -27355,7 +27491,7 @@
         </is>
       </c>
       <c r="Q28" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R28" t="n">
         <v>1</v>
@@ -27438,7 +27574,7 @@
       </c>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R29" t="n">
         <v>1</v>
@@ -27521,7 +27657,7 @@
         </is>
       </c>
       <c r="Q30" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R30" t="n">
         <v>1</v>
@@ -27596,7 +27732,7 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R31" t="n">
         <v>1</v>
@@ -27679,7 +27815,7 @@
         </is>
       </c>
       <c r="Q32" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="R32" t="n">
         <v>1</v>
@@ -27766,7 +27902,7 @@
         </is>
       </c>
       <c r="Q33" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R33" t="n">
         <v>1</v>
@@ -27853,7 +27989,7 @@
         </is>
       </c>
       <c r="Q34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R34" t="n">
         <v>1</v>
@@ -27940,7 +28076,7 @@
         </is>
       </c>
       <c r="Q35" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R35" t="n">
         <v>1</v>
@@ -28027,7 +28163,7 @@
         </is>
       </c>
       <c r="Q36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R36" t="n">
         <v>1</v>
@@ -28114,7 +28250,7 @@
         </is>
       </c>
       <c r="Q37" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R37" t="n">
         <v>1</v>
@@ -28197,7 +28333,7 @@
         </is>
       </c>
       <c r="Q38" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R38" t="n">
         <v>1</v>
@@ -28272,7 +28408,7 @@
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R39" t="n">
         <v>1</v>
@@ -28837,7 +28973,7 @@
       </c>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R46" t="n">
         <v>1</v>
@@ -28920,7 +29056,7 @@
         </is>
       </c>
       <c r="Q47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R47" t="n">
         <v>1</v>
@@ -29007,7 +29143,7 @@
         </is>
       </c>
       <c r="Q48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R48" t="n">
         <v>1</v>
@@ -29082,7 +29218,7 @@
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr"/>
       <c r="Q49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R49" t="n">
         <v>1</v>
@@ -29169,7 +29305,7 @@
         </is>
       </c>
       <c r="Q50" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R50" t="n">
         <v>1</v>
@@ -29252,7 +29388,7 @@
         </is>
       </c>
       <c r="Q51" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R51" t="n">
         <v>1</v>
@@ -29339,7 +29475,7 @@
         </is>
       </c>
       <c r="Q52" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R52" t="n">
         <v>1</v>
@@ -29426,7 +29562,7 @@
         </is>
       </c>
       <c r="Q53" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R53" t="n">
         <v>1</v>
@@ -29513,7 +29649,7 @@
         </is>
       </c>
       <c r="Q54" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R54" t="n">
         <v>1</v>
@@ -29600,7 +29736,7 @@
         </is>
       </c>
       <c r="Q55" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R55" t="n">
         <v>1</v>
@@ -29683,7 +29819,7 @@
       </c>
       <c r="P56" t="inlineStr"/>
       <c r="Q56" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R56" t="n">
         <v>1</v>
@@ -29758,7 +29894,7 @@
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr"/>
       <c r="Q57" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R57" t="n">
         <v>1</v>
@@ -29845,7 +29981,7 @@
         </is>
       </c>
       <c r="Q58" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R58" t="n">
         <v>1</v>
@@ -29932,7 +30068,7 @@
         </is>
       </c>
       <c r="Q59" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R59" t="n">
         <v>1</v>
@@ -30019,7 +30155,7 @@
         </is>
       </c>
       <c r="Q60" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R60" t="n">
         <v>1</v>
@@ -30106,7 +30242,7 @@
         </is>
       </c>
       <c r="Q61" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R61" t="n">
         <v>1</v>
@@ -30193,7 +30329,7 @@
         </is>
       </c>
       <c r="Q62" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R62" t="n">
         <v>1</v>
@@ -30276,7 +30412,7 @@
         </is>
       </c>
       <c r="Q63" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R63" t="n">
         <v>1</v>
@@ -30351,7 +30487,7 @@
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr"/>
       <c r="Q64" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="R64" t="n">
         <v>1</v>
@@ -30433,11 +30569,15 @@
         </is>
       </c>
       <c r="P65" t="inlineStr"/>
-      <c r="Q65" t="inlineStr"/>
+      <c r="Q65" t="n">
+        <v>1</v>
+      </c>
       <c r="R65" t="n">
-        <v>0</v>
-      </c>
-      <c r="S65" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S65" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -30516,11 +30656,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q66" t="inlineStr"/>
+      <c r="Q66" t="n">
+        <v>1</v>
+      </c>
       <c r="R66" t="n">
-        <v>0</v>
-      </c>
-      <c r="S66" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S66" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -30599,11 +30743,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q67" t="inlineStr"/>
+      <c r="Q67" t="n">
+        <v>1</v>
+      </c>
       <c r="R67" t="n">
-        <v>0</v>
-      </c>
-      <c r="S67" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S67" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -30678,11 +30826,15 @@
         </is>
       </c>
       <c r="P68" t="inlineStr"/>
-      <c r="Q68" t="inlineStr"/>
+      <c r="Q68" t="n">
+        <v>1</v>
+      </c>
       <c r="R68" t="n">
-        <v>0</v>
-      </c>
-      <c r="S68" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S68" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -30712,10 +30864,14 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr"/>
+          <t>22:27</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
       <c r="H69" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -30728,17 +30884,17 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>多次终点ETA一致</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -30748,12 +30904,20 @@
       </c>
       <c r="N69" t="inlineStr"/>
       <c r="O69" t="inlineStr"/>
-      <c r="P69" t="inlineStr"/>
-      <c r="Q69" t="inlineStr"/>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>多次终点ETA一致推算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="Q69" t="n">
+        <v>1</v>
+      </c>
       <c r="R69" t="n">
-        <v>0</v>
-      </c>
-      <c r="S69" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S69" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -30828,11 +30992,15 @@
         </is>
       </c>
       <c r="P70" t="inlineStr"/>
-      <c r="Q70" t="inlineStr"/>
+      <c r="Q70" t="n">
+        <v>3</v>
+      </c>
       <c r="R70" t="n">
-        <v>0</v>
-      </c>
-      <c r="S70" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S70" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -30911,11 +31079,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q71" t="inlineStr"/>
+      <c r="Q71" t="n">
+        <v>3</v>
+      </c>
       <c r="R71" t="n">
-        <v>0</v>
-      </c>
-      <c r="S71" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S71" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -30990,11 +31162,15 @@
         </is>
       </c>
       <c r="P72" t="inlineStr"/>
-      <c r="Q72" t="inlineStr"/>
+      <c r="Q72" t="n">
+        <v>3</v>
+      </c>
       <c r="R72" t="n">
-        <v>0</v>
-      </c>
-      <c r="S72" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S72" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -31069,11 +31245,15 @@
         </is>
       </c>
       <c r="P73" t="inlineStr"/>
-      <c r="Q73" t="inlineStr"/>
+      <c r="Q73" t="n">
+        <v>3</v>
+      </c>
       <c r="R73" t="n">
-        <v>0</v>
-      </c>
-      <c r="S73" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S73" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -31103,10 +31283,14 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr"/>
+          <t>23:03</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
       <c r="H74" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -31119,17 +31303,17 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>多次终点ETA一致</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -31139,12 +31323,20 @@
       </c>
       <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr"/>
-      <c r="P74" t="inlineStr"/>
-      <c r="Q74" t="inlineStr"/>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>多次终点ETA一致推算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="Q74" t="n">
+        <v>3</v>
+      </c>
       <c r="R74" t="n">
-        <v>0</v>
-      </c>
-      <c r="S74" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S74" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -31220,7 +31412,7 @@
       </c>
       <c r="P75" t="inlineStr"/>
       <c r="Q75" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R75" t="n">
         <v>1</v>
@@ -31303,7 +31495,7 @@
       </c>
       <c r="P76" t="inlineStr"/>
       <c r="Q76" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R76" t="n">
         <v>1</v>
@@ -31390,7 +31582,7 @@
         </is>
       </c>
       <c r="Q77" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R77" t="n">
         <v>1</v>
@@ -31477,7 +31669,7 @@
         </is>
       </c>
       <c r="Q78" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R78" t="n">
         <v>1</v>
@@ -31564,7 +31756,7 @@
         </is>
       </c>
       <c r="Q79" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R79" t="n">
         <v>1</v>
@@ -31647,7 +31839,7 @@
         </is>
       </c>
       <c r="Q80" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R80" t="n">
         <v>1</v>
@@ -31730,7 +31922,7 @@
       </c>
       <c r="P81" t="inlineStr"/>
       <c r="Q81" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="R81" t="n">
         <v>1</v>
@@ -31817,7 +32009,7 @@
         </is>
       </c>
       <c r="Q82" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="R82" t="n">
         <v>1</v>
@@ -31900,7 +32092,7 @@
         </is>
       </c>
       <c r="Q83" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="R83" t="n">
         <v>1</v>
@@ -31975,7 +32167,7 @@
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr"/>
       <c r="Q84" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="R84" t="n">
         <v>1</v>
@@ -32062,7 +32254,7 @@
         </is>
       </c>
       <c r="Q85" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R85" t="n">
         <v>1</v>
@@ -32149,7 +32341,7 @@
         </is>
       </c>
       <c r="Q86" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R86" t="n">
         <v>1</v>
@@ -32236,7 +32428,7 @@
         </is>
       </c>
       <c r="Q87" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R87" t="n">
         <v>1</v>
@@ -32319,7 +32511,7 @@
         </is>
       </c>
       <c r="Q88" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R88" t="n">
         <v>1</v>
@@ -32394,7 +32586,7 @@
       <c r="O89" t="inlineStr"/>
       <c r="P89" t="inlineStr"/>
       <c r="Q89" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R89" t="n">
         <v>1</v>
@@ -33470,7 +33662,7 @@
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="8" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="19" customWidth="1" min="16" max="16"/>
     <col width="8" customWidth="1" min="17" max="17"/>
@@ -34423,7 +34615,7 @@
       </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R12" t="n">
         <v>1</v>
@@ -34506,7 +34698,7 @@
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R13" t="n">
         <v>1</v>
@@ -34593,7 +34785,7 @@
         </is>
       </c>
       <c r="Q14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R14" t="n">
         <v>1</v>
@@ -34676,7 +34868,7 @@
       </c>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R15" t="n">
         <v>1</v>
@@ -35928,7 +36120,7 @@
         </is>
       </c>
       <c r="Q31" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R31" t="n">
         <v>2</v>
@@ -36011,7 +36203,7 @@
         </is>
       </c>
       <c r="Q32" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R32" t="n">
         <v>2</v>
@@ -36094,7 +36286,7 @@
         </is>
       </c>
       <c r="Q33" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R33" t="n">
         <v>2</v>
@@ -36181,7 +36373,7 @@
         </is>
       </c>
       <c r="Q34" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R34" t="n">
         <v>2</v>
@@ -36268,7 +36460,7 @@
         </is>
       </c>
       <c r="Q35" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R35" t="n">
         <v>2</v>
@@ -36343,7 +36535,7 @@
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R36" t="n">
         <v>2</v>
@@ -36430,7 +36622,7 @@
         </is>
       </c>
       <c r="Q37" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R37" t="n">
         <v>2</v>
@@ -36513,7 +36705,7 @@
         </is>
       </c>
       <c r="Q38" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R38" t="n">
         <v>2</v>
@@ -36600,7 +36792,7 @@
         </is>
       </c>
       <c r="Q39" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R39" t="n">
         <v>2</v>
@@ -36687,7 +36879,7 @@
         </is>
       </c>
       <c r="Q40" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R40" t="n">
         <v>2</v>
@@ -36770,7 +36962,7 @@
         </is>
       </c>
       <c r="Q41" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R41" t="n">
         <v>2</v>
@@ -36857,7 +37049,7 @@
         </is>
       </c>
       <c r="Q42" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R42" t="n">
         <v>1</v>
@@ -36940,7 +37132,7 @@
       </c>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R43" t="n">
         <v>1</v>
@@ -37027,7 +37219,7 @@
         </is>
       </c>
       <c r="Q44" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R44" t="n">
         <v>1</v>
@@ -37110,7 +37302,7 @@
         </is>
       </c>
       <c r="Q45" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R45" t="n">
         <v>1</v>
@@ -37193,7 +37385,7 @@
         </is>
       </c>
       <c r="Q46" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -37280,7 +37472,7 @@
         </is>
       </c>
       <c r="Q47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -37363,7 +37555,7 @@
         </is>
       </c>
       <c r="Q48" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -37450,7 +37642,7 @@
         </is>
       </c>
       <c r="Q49" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R49" t="n">
         <v>3</v>
@@ -37537,7 +37729,7 @@
         </is>
       </c>
       <c r="Q50" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -37620,7 +37812,7 @@
         </is>
       </c>
       <c r="Q51" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -37703,7 +37895,7 @@
       </c>
       <c r="P52" t="inlineStr"/>
       <c r="Q52" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R52" t="n">
         <v>1</v>
@@ -37790,7 +37982,7 @@
         </is>
       </c>
       <c r="Q53" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R53" t="n">
         <v>1</v>
@@ -37877,7 +38069,7 @@
         </is>
       </c>
       <c r="Q54" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R54" t="n">
         <v>1</v>
@@ -37960,7 +38152,7 @@
         </is>
       </c>
       <c r="Q55" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R55" t="n">
         <v>1</v>
@@ -38047,7 +38239,7 @@
         </is>
       </c>
       <c r="Q56" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R56" t="n">
         <v>1</v>
@@ -38134,7 +38326,7 @@
         </is>
       </c>
       <c r="Q57" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R57" t="n">
         <v>1</v>
@@ -38221,7 +38413,7 @@
         </is>
       </c>
       <c r="Q58" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R58" t="n">
         <v>1</v>
@@ -38304,7 +38496,7 @@
         </is>
       </c>
       <c r="Q59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R59" t="n">
         <v>1</v>
@@ -38951,11 +39143,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q67" t="inlineStr"/>
+      <c r="Q67" t="n">
+        <v>5</v>
+      </c>
       <c r="R67" t="n">
-        <v>0</v>
-      </c>
-      <c r="S67" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S67" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -39034,11 +39230,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q68" t="inlineStr"/>
+      <c r="Q68" t="n">
+        <v>5</v>
+      </c>
       <c r="R68" t="n">
-        <v>0</v>
-      </c>
-      <c r="S68" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S68" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -39074,12 +39274,12 @@
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>全程车</t>
+          <t>运行异常待查</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>未发现可靠中途折返证据</t>
+          <t>存在方向切换，但未达到提前反向80%判据</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -39102,14 +39302,26 @@
           <t>07:10</t>
         </is>
       </c>
-      <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr"/>
+      <c r="N69" s="1" t="inlineStr">
+        <is>
+          <t>长岛路张杨北路</t>
+        </is>
+      </c>
+      <c r="O69" s="1" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
       <c r="P69" t="inlineStr"/>
-      <c r="Q69" t="inlineStr"/>
+      <c r="Q69" t="n">
+        <v>5</v>
+      </c>
       <c r="R69" t="n">
-        <v>0</v>
-      </c>
-      <c r="S69" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S69" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -39139,10 +39351,14 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr"/>
+          <t>22:38</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
       <c r="H70" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -39155,17 +39371,17 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>多次终点ETA一致</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -39175,12 +39391,20 @@
       </c>
       <c r="N70" t="inlineStr"/>
       <c r="O70" t="inlineStr"/>
-      <c r="P70" t="inlineStr"/>
-      <c r="Q70" t="inlineStr"/>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>多次终点ETA一致推算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="Q70" t="n">
+        <v>5</v>
+      </c>
       <c r="R70" t="n">
-        <v>0</v>
-      </c>
-      <c r="S70" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S70" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -39256,7 +39480,7 @@
       </c>
       <c r="P71" t="inlineStr"/>
       <c r="Q71" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R71" t="n">
         <v>1</v>
@@ -39343,7 +39567,7 @@
         </is>
       </c>
       <c r="Q72" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R72" t="n">
         <v>1</v>
@@ -39426,7 +39650,7 @@
         </is>
       </c>
       <c r="Q73" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R73" t="n">
         <v>1</v>
@@ -39501,7 +39725,7 @@
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr"/>
       <c r="Q74" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R74" t="n">
         <v>1</v>
@@ -39588,13 +39812,13 @@
         </is>
       </c>
       <c r="Q75" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R75" t="n">
         <v>1</v>
       </c>
       <c r="S75" t="n">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="76">
@@ -39675,13 +39899,13 @@
         </is>
       </c>
       <c r="Q76" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R76" t="n">
         <v>1</v>
       </c>
       <c r="S76" t="n">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="77">
@@ -39712,37 +39936,33 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>20:31</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>131</t>
-        </is>
-      </c>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>全程车</t>
+          <t>运行异常待查</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>未发现可靠中途折返证据</t>
+          <t>末次同向观测已进入线路末段，存在终点漏采可能</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>末次终点ETA</t>
+          <t>证据不足</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -39750,21 +39970,29 @@
           <t>07:24</t>
         </is>
       </c>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr"/>
+      <c r="N77" s="1" t="inlineStr">
+        <is>
+          <t>康弘路康佳路（康桥卫生中心）</t>
+        </is>
+      </c>
+      <c r="O77" s="1" t="inlineStr">
+        <is>
+          <t>20:24</t>
+        </is>
+      </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>末次终点ETA推算，约±10分钟</t>
+          <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
       <c r="Q77" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R77" t="n">
         <v>1</v>
       </c>
       <c r="S77" t="n">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="78">
@@ -39795,10 +40023,14 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr"/>
+          <t>22:58</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
       <c r="H78" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -39811,17 +40043,17 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>末次终点ETA</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -39831,15 +40063,19 @@
       </c>
       <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr"/>
-      <c r="P78" t="inlineStr"/>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>末次终点ETA推算，约±15分钟</t>
+        </is>
+      </c>
       <c r="Q78" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R78" t="n">
         <v>1</v>
       </c>
       <c r="S78" t="n">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="79">
@@ -40406,7 +40642,7 @@
         </is>
       </c>
       <c r="Q85" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R85" t="n">
         <v>1</v>
@@ -40493,7 +40729,7 @@
         </is>
       </c>
       <c r="Q86" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R86" t="n">
         <v>1</v>
@@ -40576,7 +40812,7 @@
       </c>
       <c r="P87" t="inlineStr"/>
       <c r="Q87" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R87" t="n">
         <v>1</v>
@@ -40659,7 +40895,7 @@
         </is>
       </c>
       <c r="Q88" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R88" t="n">
         <v>1</v>
@@ -40746,7 +40982,7 @@
         </is>
       </c>
       <c r="Q89" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R89" t="n">
         <v>1</v>
@@ -40829,7 +41065,7 @@
         </is>
       </c>
       <c r="Q90" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R90" t="n">
         <v>1</v>
@@ -40916,7 +41152,7 @@
         </is>
       </c>
       <c r="Q91" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R91" t="n">
         <v>1</v>
@@ -41003,7 +41239,7 @@
         </is>
       </c>
       <c r="Q92" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R92" t="n">
         <v>1</v>
@@ -41078,7 +41314,7 @@
       <c r="O93" t="inlineStr"/>
       <c r="P93" t="inlineStr"/>
       <c r="Q93" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R93" t="n">
         <v>1</v>
@@ -41481,7 +41717,7 @@
         </is>
       </c>
       <c r="Q98" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R98" t="n">
         <v>1</v>
@@ -41564,7 +41800,7 @@
         </is>
       </c>
       <c r="Q99" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R99" t="n">
         <v>1</v>
@@ -41651,7 +41887,7 @@
         </is>
       </c>
       <c r="Q100" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R100" t="n">
         <v>1</v>
@@ -41738,7 +41974,7 @@
         </is>
       </c>
       <c r="Q101" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R101" t="n">
         <v>1</v>
@@ -41825,7 +42061,7 @@
         </is>
       </c>
       <c r="Q102" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R102" t="n">
         <v>1</v>
@@ -41908,7 +42144,7 @@
         </is>
       </c>
       <c r="Q103" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R103" t="n">
         <v>1</v>
@@ -41995,7 +42231,7 @@
         </is>
       </c>
       <c r="Q104" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R104" t="n">
         <v>1</v>
@@ -42078,7 +42314,7 @@
       </c>
       <c r="P105" t="inlineStr"/>
       <c r="Q105" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R105" t="n">
         <v>1</v>
@@ -43419,11 +43655,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
+      <c r="Q13" t="n">
+        <v>1</v>
+      </c>
       <c r="R13" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S13" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -43502,11 +43742,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
+      <c r="Q14" t="n">
+        <v>1</v>
+      </c>
       <c r="R14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S14" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -43585,11 +43829,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
+      <c r="Q15" t="n">
+        <v>1</v>
+      </c>
       <c r="R15" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S15" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -43668,11 +43916,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
+      <c r="Q16" t="n">
+        <v>1</v>
+      </c>
       <c r="R16" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S16" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -43751,11 +44003,15 @@
           <t>存在终点ETA，但运行轨迹仍需复核</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
+      <c r="Q17" t="n">
+        <v>1</v>
+      </c>
       <c r="R17" t="n">
-        <v>0</v>
-      </c>
-      <c r="S17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S17" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -43830,11 +44086,15 @@
         </is>
       </c>
       <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
+      <c r="Q18" t="n">
+        <v>1</v>
+      </c>
       <c r="R18" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S18" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -43864,10 +44124,14 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>22:18</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -43880,17 +44144,17 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点近站ETA</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -43900,12 +44164,20 @@
       </c>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>终点近站ETA推算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
+        <v>1</v>
+      </c>
       <c r="R19" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S19" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -45048,7 +45320,7 @@
         </is>
       </c>
       <c r="Q33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R33" t="n">
         <v>1</v>
@@ -45135,7 +45407,7 @@
         </is>
       </c>
       <c r="Q34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R34" t="n">
         <v>1</v>
@@ -45222,7 +45494,7 @@
         </is>
       </c>
       <c r="Q35" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R35" t="n">
         <v>1</v>
@@ -45309,7 +45581,7 @@
         </is>
       </c>
       <c r="Q36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R36" t="n">
         <v>1</v>
@@ -45396,7 +45668,7 @@
         </is>
       </c>
       <c r="Q37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R37" t="n">
         <v>1</v>
@@ -45479,7 +45751,7 @@
         </is>
       </c>
       <c r="Q38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R38" t="n">
         <v>1</v>
@@ -45554,7 +45826,7 @@
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R39" t="n">
         <v>1</v>
@@ -45641,7 +45913,7 @@
         </is>
       </c>
       <c r="Q40" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R40" t="n">
         <v>1</v>
@@ -45728,7 +46000,7 @@
         </is>
       </c>
       <c r="Q41" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R41" t="n">
         <v>1</v>
@@ -45815,7 +46087,7 @@
         </is>
       </c>
       <c r="Q42" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R42" t="n">
         <v>1</v>
@@ -45902,7 +46174,7 @@
         </is>
       </c>
       <c r="Q43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R43" t="n">
         <v>1</v>
@@ -45989,7 +46261,7 @@
         </is>
       </c>
       <c r="Q44" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R44" t="n">
         <v>1</v>
@@ -46072,7 +46344,7 @@
         </is>
       </c>
       <c r="Q45" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R45" t="n">
         <v>1</v>
@@ -46147,7 +46419,7 @@
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R46" t="n">
         <v>1</v>
@@ -46471,7 +46743,7 @@
         </is>
       </c>
       <c r="Q50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R50" t="n">
         <v>1</v>
@@ -46558,7 +46830,7 @@
         </is>
       </c>
       <c r="Q51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R51" t="n">
         <v>1</v>
@@ -46641,7 +46913,7 @@
         </is>
       </c>
       <c r="Q52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R52" t="n">
         <v>1</v>
@@ -46728,7 +47000,7 @@
         </is>
       </c>
       <c r="Q53" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R53" t="n">
         <v>1</v>
@@ -46815,7 +47087,7 @@
         </is>
       </c>
       <c r="Q54" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R54" t="n">
         <v>1</v>
@@ -46902,7 +47174,7 @@
         </is>
       </c>
       <c r="Q55" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R55" t="n">
         <v>1</v>
@@ -46985,7 +47257,7 @@
         </is>
       </c>
       <c r="Q56" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R56" t="n">
         <v>1</v>
@@ -47072,7 +47344,7 @@
         </is>
       </c>
       <c r="Q57" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R57" t="n">
         <v>1</v>
@@ -47159,7 +47431,7 @@
         </is>
       </c>
       <c r="Q58" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R58" t="n">
         <v>1</v>
@@ -47246,7 +47518,7 @@
         </is>
       </c>
       <c r="Q59" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R59" t="n">
         <v>1</v>
@@ -47333,7 +47605,7 @@
         </is>
       </c>
       <c r="Q60" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R60" t="n">
         <v>1</v>
@@ -47420,7 +47692,7 @@
         </is>
       </c>
       <c r="Q61" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R61" t="n">
         <v>1</v>
@@ -47503,7 +47775,7 @@
         </is>
       </c>
       <c r="Q62" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R62" t="n">
         <v>1</v>
@@ -47578,7 +47850,7 @@
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr"/>
       <c r="Q63" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R63" t="n">
         <v>1</v>
@@ -47665,7 +47937,7 @@
         </is>
       </c>
       <c r="Q64" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R64" t="n">
         <v>1</v>
@@ -47752,7 +48024,7 @@
         </is>
       </c>
       <c r="Q65" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R65" t="n">
         <v>1</v>
@@ -47839,7 +48111,7 @@
         </is>
       </c>
       <c r="Q66" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R66" t="n">
         <v>1</v>
@@ -47926,7 +48198,7 @@
         </is>
       </c>
       <c r="Q67" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R67" t="n">
         <v>1</v>
@@ -48013,7 +48285,7 @@
         </is>
       </c>
       <c r="Q68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R68" t="n">
         <v>1</v>
@@ -48096,7 +48368,7 @@
         </is>
       </c>
       <c r="Q69" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R69" t="n">
         <v>1</v>
@@ -48171,7 +48443,7 @@
       <c r="O70" t="inlineStr"/>
       <c r="P70" t="inlineStr"/>
       <c r="Q70" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R70" t="n">
         <v>1</v>
@@ -48752,7 +49024,7 @@
         </is>
       </c>
       <c r="Q77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R77" t="n">
         <v>1</v>
@@ -48839,7 +49111,7 @@
         </is>
       </c>
       <c r="Q78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R78" t="n">
         <v>1</v>
@@ -48926,7 +49198,7 @@
         </is>
       </c>
       <c r="Q79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R79" t="n">
         <v>1</v>
@@ -49013,7 +49285,7 @@
         </is>
       </c>
       <c r="Q80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R80" t="n">
         <v>1</v>
@@ -49100,7 +49372,7 @@
         </is>
       </c>
       <c r="Q81" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R81" t="n">
         <v>1</v>
@@ -49183,7 +49455,7 @@
       </c>
       <c r="P82" t="inlineStr"/>
       <c r="Q82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R82" t="n">
         <v>1</v>
@@ -49266,7 +49538,7 @@
         </is>
       </c>
       <c r="Q83" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R83" t="n">
         <v>1</v>
@@ -49341,7 +49613,7 @@
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr"/>
       <c r="Q84" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R84" t="n">
         <v>1</v>

</xml_diff>